<commit_message>
Standaard toetsduur 10 min (één slot), TTV 15 min; voorbeeld met studenten na de pauze
</commit_message>
<xml_diff>
--- a/voorbeeld/Voorbeeld rooster.xlsx
+++ b/voorbeeld/Voorbeeld rooster.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1079,7 +1079,7 @@
         <v>46128</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.375</v>
+        <v>0.4305555555555556</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
         <v>46128</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.3819444444444444</v>
+        <v>0.4375</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         <v>46128</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.3888888888888889</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1163,7 +1163,7 @@
         <v>46128</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.4513888888888889</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1191,7 +1191,7 @@
         <v>46128</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.4027777777777778</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
         <v>46128</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.4097222222222222</v>
+        <v>0.4652777777777778</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         <v>46128</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.4722222222222222</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
         <v>46128</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.4236111111111111</v>
+        <v>0.4791666666666667</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1303,7 +1303,7 @@
         <v>46128</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.4305555555555556</v>
+        <v>0.4861111111111111</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         <v>46128</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0.4375</v>
+        <v>0.4930555555555556</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1359,7 +1359,7 @@
         <v>46128</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.5</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         <v>46128</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.4513888888888889</v>
+        <v>0.5069444444444444</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
         <v>46128</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.4583333333333333</v>
+        <v>0.5138888888888888</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1443,7 +1443,7 @@
         <v>46128</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>0.4652777777777778</v>
+        <v>0.5208333333333334</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1471,26 +1471,26 @@
         <v>46128</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0.4722222222222222</v>
+        <v>0.4305555555555556</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>XY</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Gesprek</t>
+          <t>Anamnese</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>NN</t>
         </is>
       </c>
     </row>
@@ -1499,26 +1499,26 @@
         <v>46128</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>0.4791666666666667</v>
+        <v>0.4375</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>XY</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Gesprek</t>
+          <t>Anamnese</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>NN</t>
         </is>
       </c>
     </row>
@@ -1527,26 +1527,26 @@
         <v>46128</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0.4861111111111111</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>XY</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Gesprek</t>
+          <t>Anamnese</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>NN</t>
         </is>
       </c>
     </row>
@@ -1555,26 +1555,26 @@
         <v>46128</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>0.4930555555555556</v>
+        <v>0.4513888888888889</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>XY</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Gesprek</t>
+          <t>Anamnese</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>NN</t>
         </is>
       </c>
     </row>
@@ -1583,26 +1583,26 @@
         <v>46128</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>0.5</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>XY</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Gesprek</t>
+          <t>Anamnese</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>NN</t>
         </is>
       </c>
     </row>
@@ -1611,26 +1611,26 @@
         <v>46128</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0.5069444444444444</v>
+        <v>0.4652777777777778</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>XY</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Gesprek</t>
+          <t>Anamnese</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>NN</t>
         </is>
       </c>
     </row>
@@ -1639,26 +1639,26 @@
         <v>46128</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>0.5138888888888888</v>
+        <v>0.4722222222222222</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>XY</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Gesprek</t>
+          <t>Anamnese</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>NN</t>
         </is>
       </c>
     </row>
@@ -1667,26 +1667,26 @@
         <v>46128</v>
       </c>
       <c r="B23" s="3" t="n">
-        <v>0.5208333333333334</v>
+        <v>0.4791666666666667</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>XY</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Gesprek</t>
+          <t>Anamnese</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>NN</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1695,7 @@
         <v>46128</v>
       </c>
       <c r="B24" s="3" t="n">
-        <v>0.375</v>
+        <v>0.4861111111111111</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
         <v>46128</v>
       </c>
       <c r="B25" s="3" t="n">
-        <v>0.3819444444444444</v>
+        <v>0.4930555555555556</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1751,7 +1751,7 @@
         <v>46128</v>
       </c>
       <c r="B26" s="3" t="n">
-        <v>0.3888888888888889</v>
+        <v>0.5</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
         <v>46128</v>
       </c>
       <c r="B27" s="3" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.5069444444444444</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
         <v>46128</v>
       </c>
       <c r="B28" s="3" t="n">
-        <v>0.4027777777777778</v>
+        <v>0.5138888888888888</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1835,7 +1835,7 @@
         <v>46128</v>
       </c>
       <c r="B29" s="3" t="n">
-        <v>0.4097222222222222</v>
+        <v>0.5208333333333334</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1853,454 +1853,6 @@
         </is>
       </c>
       <c r="F29" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B31" s="3" t="n">
-        <v>0.4236111111111111</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B32" s="3" t="n">
-        <v>0.4305555555555556</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B33" s="3" t="n">
-        <v>0.4375</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B34" s="3" t="n">
-        <v>0.4444444444444444</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B35" s="3" t="n">
-        <v>0.4513888888888889</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B36" s="3" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B37" s="3" t="n">
-        <v>0.4652777777777778</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B38" s="3" t="n">
-        <v>0.4722222222222222</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B39" s="3" t="n">
-        <v>0.4791666666666667</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B40" s="3" t="n">
-        <v>0.4861111111111111</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B41" s="3" t="n">
-        <v>0.4930555555555556</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B43" s="3" t="n">
-        <v>0.5069444444444444</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B44" s="3" t="n">
-        <v>0.5138888888888888</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>NN</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B45" s="3" t="n">
-        <v>0.5208333333333334</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Anamnese</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
         <is>
           <t>NN</t>
         </is>
@@ -5408,11 +4960,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Duur van een gewone toets in jaar 1.</t>
+          <t>Duur van een gewone toets in jaar 1 (= één slot van 10 minuten).</t>
         </is>
       </c>
     </row>
@@ -5423,7 +4975,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -5438,7 +4990,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -5453,7 +5005,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Instellingenpagina voor bijna alles, modulaire app (thema/onderdelen/uitvoer), nieuw ontwerp, PDF voor docenten, sjabloon
</commit_message>
<xml_diff>
--- a/voorbeeld/Voorbeeld rooster.xlsx
+++ b/voorbeeld/Voorbeeld rooster.xlsx
@@ -4913,12 +4913,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Studiejaar van deze toets (1 of 2); bepaalt welke toetsduur hieronder geldt.</t>
+          <t>Studiejaar van deze toets; bepaalt welke duur hieronder geldt.</t>
         </is>
       </c>
     </row>
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Duur van een gewone toets in jaar 1 (= één slot van 10 minuten).</t>
+          <t>Gewone toets in jaar 1 (10 min = één slot).</t>
         </is>
       </c>
     </row>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Duur voor studenten met TTV (toegestane tijdverlenging) in jaar 1.</t>
+          <t>Toets met tijdverlenging in jaar 1.</t>
         </is>
       </c>
     </row>
@@ -4994,7 +4994,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Duur van een gewone toets in jaar 2 (pas aan: jaar 2 heeft een andere tijd).</t>
+          <t>Gewone toets in jaar 2.</t>
         </is>
       </c>
     </row>
@@ -5009,7 +5009,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Duur voor studenten met TTV in jaar 2.</t>
+          <t>Toets met tijdverlenging in jaar 2.</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Begin van de pauze (bijv. 12:00). Leeg = geen pauze.</t>
+          <t>Begin van de pauze, bijv. 12:00.</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,280 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Einde van de pauze (bijv. 12:30). Leeg = geen pauze.</t>
+          <t>Einde van de pauze, bijv. 12:30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Casus na pauze gebruiken</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Slots na de pauze krijgen de casus uit de kolom 'Casus na pauze'. Keuzes: Ja / Nee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TTV-plaatsing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Eind van blok vóór pauze</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Waar TTV-studenten bij voorkeur komen. Aan het eind van het blok valt de extra tijd in de pauze. Keuzes: Eind van blok vóór pauze / Zo vroeg mogelijk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TTV-studenten eerst inroosteren</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Geeft TTV-studenten als eerste een plek, zodat de beste plekken voor hen vrij zijn. Keuzes: Ja / Nee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Namen deels vergelijken</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>‘Ann’ sluit dan ook ‘Anneke’ uit. Vangt spelfouten op, maar kan te veel uitsluiten. Keuzes: Ja / Nee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Andere beoordelaar dan 1e kans</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Voorkeur</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Verplicht: lukt het niet, dan wordt de student niet ingeroosterd. Keuzes: Voorkeur / Verplicht / Maakt niet uit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Andere casus dan 1e kans</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Voorkeur</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Verplicht: lukt het niet, dan wordt de student niet ingeroosterd. Keuzes: Voorkeur / Verplicht / Maakt niet uit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rooster sorteren op</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Lokaal, dan tijd</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Volgorde van het volledige rooster (altijd eerst per datum). Keuzes: Lokaal, dan tijd / Tijd, dan lokaal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Uitdraai sorteren op</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Achternaam</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Volgorde van de uitdraai voor studenten. Keuzes: Achternaam / Tijd / Lokaal, dan tijd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Datum op uitdraai</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Nee: alleen de begintijd (handig als alles op één dag is). Keuzes: Ja / Nee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Blad studenten</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Studenten</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Blad slots eerste kans</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Slots_Kans1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Blad slots herkansing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Slots_Her</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Blad beoordelaars</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Beoordelaars</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Blad simucliënten</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Simu</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Blad rooster eerste kans</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Rooster_Kans1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Blad rooster herkansing</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Rooster_Her</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Blad uitdraai eerste kans</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Uitdraai_Kans1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Blad uitdraai herkansing</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Uitdraai_Her</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Blad meldingen</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Meldingen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Beoordelaars met tijden in de cel (tot/vanaf/10.00-12.00), Beoordelaar 3+, ruilen met controle op dubbel inzetten; lokalen evenredig vullen; melding per lokaal dat niemand krijgt; voorbeeldnamen vervangen
</commit_message>
<xml_diff>
--- a/voorbeeld/Voorbeeld rooster.xlsx
+++ b/voorbeeld/Voorbeeld rooster.xlsx
@@ -3381,7 +3381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -3458,218 +3458,218 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jaar</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
+          <t>Lokalen vullen</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Evenredig</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Studiejaar van deze toets; bepaalt welke duur hieronder geldt.</t>
+          <t>Evenredig: op elk tijdstip eerst het lokaal met de minste studenten, zodat elk lokaal (en elke beoordelaar) ongeveer evenveel krijgt, ook als er minder simu's dan lokalen zijn. Op volgorde: eerst de bovenste lokalen. Keuzes: Evenredig / Op volgorde.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Toetsduur jaar 1 (min)</t>
+          <t>Jaar</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gewone toets in jaar 1.</t>
+          <t>Studiejaar van deze toets; bepaalt welke duur hieronder geldt.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TTV-toetsduur jaar 1 (min)</t>
+          <t>Toetsduur jaar 1 (min)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Toets met tijdverlenging in jaar 1.</t>
+          <t>Gewone toets in jaar 1.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Toetsduur jaar 2 (min)</t>
+          <t>TTV-toetsduur jaar 1 (min)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Gewone toets in jaar 2.</t>
+          <t>Toets met tijdverlenging in jaar 1.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TTV-toetsduur jaar 2 (min)</t>
+          <t>Toetsduur jaar 2 (min)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Toets met tijdverlenging in jaar 2.</t>
+          <t>Gewone toets in jaar 2.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Pauzes</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>11:15-11:40, 13:00-13:55, 15:15-15:40</t>
-        </is>
+          <t>TTV-toetsduur jaar 2 (min)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>20</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Van-tot, meerdere gescheiden door een komma. Leeg = geen pauze.</t>
+          <t>Toets met tijdverlenging in jaar 2.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Casus na pauze</t>
+          <t>Pauzes</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Na pauze 1</t>
+          <t>11:15-11:40, 13:00-13:55, 15:15-15:40</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wanneer slots de casus uit de kolom 'Casus na pauze' krijgen (alleen als die kolom is ingevuld). Keuzes: Nee / Na pauze 1 / Na pauze 2 / Na pauze 3 / Na elke pauze afwisselen.</t>
+          <t>Van-tot, meerdere gescheiden door een komma. Leeg = geen pauze.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TTV-plaatsing</t>
+          <t>Casus na pauze</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Eind van blok vóór pauze</t>
+          <t>Na pauze 1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Waar TTV-studenten bij voorkeur komen. Aan het eind van een blok valt de extra tijd in de pauze. Keuzes: Eind van blok vóór pauze / Zo vroeg mogelijk.</t>
+          <t>Wanneer slots de casus uit de kolom 'Casus na pauze' krijgen (alleen als die kolom is ingevuld). Keuzes: Nee / Na pauze 1 / Na pauze 2 / Na pauze 3 / Na elke pauze afwisselen.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TTV-studenten eerst inroosteren</t>
+          <t>TTV-plaatsing</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Eind van blok vóór pauze</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Geeft TTV-studenten als eerste een plek, zodat de beste plekken voor hen vrij zijn. Keuzes: Ja / Nee.</t>
+          <t>Waar TTV-studenten bij voorkeur komen. Aan het eind van een blok valt de extra tijd in de pauze. Keuzes: Eind van blok vóór pauze / Zo vroeg mogelijk.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Middag begint om</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>12:00</t>
+          <t>TTV-studenten eerst inroosteren</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Ja</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Grens tussen voorkeur ochtend en middag.</t>
+          <t>Geeft TTV-studenten als eerste een plek, zodat de beste plekken voor hen vrij zijn. Keuzes: Ja / Nee.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Simu's rouleren per blok</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Ja</t>
+          <t>Middag begint om</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Na elke pauze schuift elke simucliënt een lokaal door. Nee: iedere simu blijft in hetzelfde lokaal. Keuzes: Ja / Nee.</t>
+          <t>Grens tussen voorkeur ochtend en middag.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Namen deels vergelijken</t>
+          <t>Simu's wisselen van lokaal</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Na elke pauze</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>‘Ann’ sluit dan ook ‘Anneke’ uit. Vangt spelfouten op, maar kan te veel uitsluiten. Keuzes: Ja / Nee.</t>
+          <t>Na elke pauze of na elke toets schuift elke simucliënt een lokaal door, zodat niemand de hele dag bij dezelfde toets zit. Nee: iedere simu blijft in hetzelfde lokaal. Keuzes: Na elke pauze / Na elke toets / Nee.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Andere beoordelaar dan 1e kans</t>
+          <t>Namen deels vergelijken</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Voorkeur</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Verplicht: lukt het niet, dan wordt de student niet ingeroosterd. Keuzes: Voorkeur / Verplicht / Maakt niet uit.</t>
+          <t>‘Ann’ sluit dan ook ‘Anneke’ uit. Vangt spelfouten op, maar kan te veel uitsluiten. Keuzes: Ja / Nee.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Andere casus dan 1e kans</t>
+          <t>Andere beoordelaar dan 1e kans</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3686,210 +3686,227 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Vrije plekken tonen</t>
+          <t>Andere casus dan 1e kans</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Voorkeur</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Lege maar bruikbare plekken als 'Vrije plek' in het volledige rooster (nooit op de uitdraai of in de PDF's). Keuzes: Ja / Nee.</t>
+          <t>Verplicht: lukt het niet, dan wordt de student niet ingeroosterd. Keuzes: Voorkeur / Verplicht / Maakt niet uit.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Rooster sorteren op</t>
+          <t>Vrije plekken tonen</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Lokaal, dan tijd</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Volgorde van het volledige rooster (altijd eerst per datum). Keuzes: Lokaal, dan tijd / Tijd, dan lokaal.</t>
+          <t>Lege maar bruikbare plekken als 'Vrije plek' in het volledige rooster (nooit op de uitdraai of in de PDF's). Keuzes: Ja / Nee.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Uitdraai sorteren op</t>
+          <t>Rooster sorteren op</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Achternaam</t>
+          <t>Lokaal, dan tijd</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Volgorde van de uitdraai voor studenten. Keuzes: Achternaam / Tijd / Lokaal, dan tijd.</t>
+          <t>Volgorde van het volledige rooster (altijd eerst per datum). Keuzes: Lokaal, dan tijd / Tijd, dan lokaal.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Datum op uitdraai</t>
+          <t>Uitdraai sorteren op</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Achternaam</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Nee: alleen de begintijd (handig als alles op één dag is). Keuzes: Ja / Nee.</t>
+          <t>Volgorde van de uitdraai voor studenten. Keuzes: Achternaam / Tijd / Lokaal, dan tijd.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Blad studenten</t>
+          <t>Datum op uitdraai</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Studenten</t>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Nee: alleen de begintijd (handig als alles op één dag is). Keuzes: Ja / Nee.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Blad toetsdag eerste kans</t>
+          <t>Blad studenten</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Toetsdag_Kans1</t>
+          <t>Studenten</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Blad toetsdag herkansing</t>
+          <t>Blad toetsdag eerste kans</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Toetsdag_Her</t>
+          <t>Toetsdag_Kans1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Blad simucliënten</t>
+          <t>Blad toetsdag herkansing</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Simu</t>
+          <t>Toetsdag_Her</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Blad slots eerste kans (oud)</t>
+          <t>Blad simucliënten</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Slots_Kans1</t>
+          <t>Simu</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Blad slots herkansing (oud)</t>
+          <t>Blad slots eerste kans (oud)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Slots_Her</t>
+          <t>Slots_Kans1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Blad beoordelaars (oud)</t>
+          <t>Blad slots herkansing (oud)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Beoordelaars</t>
+          <t>Slots_Her</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Blad rooster eerste kans</t>
+          <t>Blad beoordelaars (oud)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Rooster_Kans1</t>
+          <t>Beoordelaars</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Blad rooster herkansing</t>
+          <t>Blad rooster eerste kans</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Rooster_Her</t>
+          <t>Rooster_Kans1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Blad uitdraai eerste kans</t>
+          <t>Blad rooster herkansing</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Uitdraai_Kans1</t>
+          <t>Rooster_Her</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Blad uitdraai herkansing</t>
+          <t>Blad uitdraai eerste kans</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Uitdraai_Her</t>
+          <t>Uitdraai_Kans1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Blad uitdraai herkansing</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Uitdraai_Her</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Blad meldingen</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Meldingen</t>
         </is>

</xml_diff>

<commit_message>
Teksten eenvoudiger (README, REGELS, Hulp); voorbeeldwerkmap met kolommen Van/Tot en Vast lokaal/Kan spelen
</commit_message>
<xml_diff>
--- a/voorbeeld/Voorbeeld rooster.xlsx
+++ b/voorbeeld/Voorbeeld rooster.xlsx
@@ -2932,7 +2932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2941,8 +2941,11 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2978,12 +2981,27 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Van</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Beoordelaar 2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Wissel om</t>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Van 2</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Tot 2</t>
         </is>
       </c>
     </row>
@@ -3111,12 +3129,17 @@
           <t>Eef</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Fien</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
@@ -3133,7 +3156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3142,8 +3165,11 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3179,12 +3205,27 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Van</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Beoordelaar 2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Wissel om</t>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Van 2</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Tot 2</t>
         </is>
       </c>
     </row>
@@ -3254,13 +3295,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3282,6 +3325,16 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Tot</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Vast lokaal</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Kan spelen</t>
         </is>
       </c>
     </row>

</xml_diff>